<commit_message>
Add fix config load
</commit_message>
<xml_diff>
--- a/data/ubp.xlsx
+++ b/data/ubp.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,6 +456,99 @@
         <is>
           <t>linkName</t>
         </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>dealSize</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>propensityToWin</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>isStrategic</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>&lt; $100k</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Test 2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>&lt; $100k</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K3" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>